<commit_message>
docs: 테이블 명세서에 users.avatar_key 추가
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AcRn9gV7oGMnFFhj3kFFXF
</commit_message>
<xml_diff>
--- a/docs/MeerKit_테이블명세서.xlsx
+++ b/docs/MeerKit_테이블명세서.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="관계" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'컬럼 명세'!$A$1:$L$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'컬럼 명세'!$A$1:$L$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -513,6 +513,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -533,7 +534,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>5aeec7c9a772</t>
+          <t>d129bc5cc95b</t>
         </is>
       </c>
     </row>
@@ -545,7 +546,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>main bae1b41 (PR #13 병합)</t>
+          <t>main fe80117 (PR #29 병합)</t>
         </is>
       </c>
     </row>
@@ -557,7 +558,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-25 (2026-10-27 users.avatar_key 추가)</t>
         </is>
       </c>
     </row>
@@ -585,6 +586,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -639,7 +641,7 @@
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13">
@@ -810,7 +812,7 @@
         </is>
       </c>
       <c r="E20" s="9" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -824,7 +826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1603,12 +1605,12 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>email_verified_at</t>
+          <t>avatar_key</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>TIMESTAMPTZ</t>
+          <t>VARCHAR(200)</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
@@ -1616,14 +1618,14 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G18" s="11" t="inlineStr"/>
-      <c r="H18" s="10" t="inlineStr"/>
-      <c r="I18" s="11" t="inlineStr"/>
-      <c r="J18" s="10" t="inlineStr"/>
-      <c r="K18" s="11" t="inlineStr"/>
+      <c r="G18" s="11" t="n"/>
+      <c r="H18" s="10" t="n"/>
+      <c r="I18" s="11" t="n"/>
+      <c r="J18" s="10" t="n"/>
+      <c r="K18" s="11" t="n"/>
       <c r="L18" s="11" t="inlineStr">
         <is>
-          <t>이메일 인증 완료 시각 (NULL이면 미인증)</t>
+          <t>프로필 이미지 파일의 저장소 key (avatars/&lt;무작위&gt;.webp). 교체·삭제·파기 때 이전 파일을 지우는 데 씀. 파일은 Supabase Storage 버킷 meerkit-public에 있음</t>
         </is>
       </c>
     </row>
@@ -1643,31 +1645,27 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>failed_login_count</t>
+          <t>email_verified_at</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>INTEGER</t>
+          <t>TIMESTAMPTZ</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G19" s="11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr"/>
       <c r="H19" s="10" t="inlineStr"/>
       <c r="I19" s="11" t="inlineStr"/>
       <c r="J19" s="10" t="inlineStr"/>
       <c r="K19" s="11" t="inlineStr"/>
       <c r="L19" s="11" t="inlineStr">
         <is>
-          <t>연속 로그인 실패 횟수 (성공·잠금 시 0으로 초기화)</t>
+          <t>이메일 인증 완료 시각 (NULL이면 미인증)</t>
         </is>
       </c>
     </row>
@@ -1687,27 +1685,31 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>locked_until</t>
+          <t>failed_login_count</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>TIMESTAMPTZ</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G20" s="11" t="inlineStr"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="H20" s="10" t="inlineStr"/>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="10" t="inlineStr"/>
       <c r="K20" s="11" t="inlineStr"/>
       <c r="L20" s="11" t="inlineStr">
         <is>
-          <t>로그인 잠금 해제 시각 (5회 실패 → 5분)</t>
+          <t>연속 로그인 실패 횟수 (성공·잠금 시 0으로 초기화)</t>
         </is>
       </c>
     </row>
@@ -1727,7 +1729,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>last_login_at</t>
+          <t>locked_until</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -1747,7 +1749,7 @@
       <c r="K21" s="11" t="inlineStr"/>
       <c r="L21" s="11" t="inlineStr">
         <is>
-          <t>마지막 로그인 시각</t>
+          <t>로그인 잠금 해제 시각 (5회 실패 → 5분)</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1769,7 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>password_changed_at</t>
+          <t>last_login_at</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -1787,7 +1789,7 @@
       <c r="K22" s="11" t="inlineStr"/>
       <c r="L22" s="11" t="inlineStr">
         <is>
-          <t>비밀번호 변경 시각. 이전에 발급된 토큰은 거부</t>
+          <t>마지막 로그인 시각</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1809,7 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>deactivated_at</t>
+          <t>password_changed_at</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
@@ -1827,7 +1829,7 @@
       <c r="K23" s="11" t="inlineStr"/>
       <c r="L23" s="11" t="inlineStr">
         <is>
-          <t>탈퇴(또는 관리자 삭제) 시각. 보관 기간 계산 기준</t>
+          <t>비밀번호 변경 시각. 이전에 발급된 토큰은 거부</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1849,7 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>deleted_at</t>
+          <t>deactivated_at</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -1867,55 +1869,47 @@
       <c r="K24" s="11" t="inlineStr"/>
       <c r="L24" s="11" t="inlineStr">
         <is>
+          <t>탈퇴(또는 관리자 삭제) 시각. 보관 기간 계산 기준</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>회원</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>deleted_at</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr"/>
+      <c r="H25" s="10" t="inlineStr"/>
+      <c r="I25" s="11" t="inlineStr"/>
+      <c r="J25" s="10" t="inlineStr"/>
+      <c r="K25" s="11" t="inlineStr"/>
+      <c r="L25" s="11" t="inlineStr">
+        <is>
           <t>개인정보 파기 시각 (탈퇴 후 365일, purge 명령)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>roles</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>역할</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>자동 증가</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="I25" s="8" t="inlineStr"/>
-      <c r="J25" s="6" t="inlineStr"/>
-      <c r="K25" s="8" t="inlineStr"/>
-      <c r="L25" s="8" t="inlineStr">
-        <is>
-          <t>역할 번호 (1 MASTER, 2 OWNER, 3 VIEWER, 4 WRITER)</t>
         </is>
       </c>
     </row>
@@ -1935,12 +1929,12 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>VARCHAR(30)</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -1948,22 +1942,22 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G26" s="8" t="inlineStr"/>
-      <c r="H26" s="6" t="inlineStr"/>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>자동 증가</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="I26" s="8" t="inlineStr"/>
-      <c r="J26" s="6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K26" s="8" t="inlineStr">
-        <is>
-          <t>UNIQUE roles_code_key</t>
-        </is>
-      </c>
+      <c r="J26" s="6" t="inlineStr"/>
+      <c r="K26" s="8" t="inlineStr"/>
       <c r="L26" s="8" t="inlineStr">
         <is>
-          <t>역할 코드. 코드에서 비교하는 값</t>
+          <t>역할 번호 (1 MASTER, 2 OWNER, 3 VIEWER, 4 WRITER)</t>
         </is>
       </c>
     </row>
@@ -1983,12 +1977,12 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>VARCHAR(50)</t>
+          <t>VARCHAR(30)</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -1999,59 +1993,59 @@
       <c r="G27" s="8" t="inlineStr"/>
       <c r="H27" s="6" t="inlineStr"/>
       <c r="I27" s="8" t="inlineStr"/>
-      <c r="J27" s="6" t="inlineStr"/>
-      <c r="K27" s="8" t="inlineStr"/>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K27" s="8" t="inlineStr">
+        <is>
+          <t>UNIQUE roles_code_key</t>
+        </is>
+      </c>
       <c r="L27" s="8" t="inlineStr">
         <is>
+          <t>역할 코드. 코드에서 비교하는 값</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>roles</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>역할</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>VARCHAR(50)</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr"/>
+      <c r="H28" s="6" t="inlineStr"/>
+      <c r="I28" s="8" t="inlineStr"/>
+      <c r="J28" s="6" t="inlineStr"/>
+      <c r="K28" s="8" t="inlineStr"/>
+      <c r="L28" s="8" t="inlineStr">
+        <is>
           <t>화면 표시용 설명</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>user_roles</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="inlineStr">
-        <is>
-          <t>회원-역할 연결</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="inlineStr">
-        <is>
-          <t>user_id</t>
-        </is>
-      </c>
-      <c r="E28" s="11" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="F28" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G28" s="11" t="inlineStr"/>
-      <c r="H28" s="10" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr">
-        <is>
-          <t>users.id (ON DELETE CASCADE)</t>
-        </is>
-      </c>
-      <c r="J28" s="10" t="inlineStr"/>
-      <c r="K28" s="11" t="inlineStr"/>
-      <c r="L28" s="11" t="inlineStr">
-        <is>
-          <t>회원 번호</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2065,7 @@
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>role_id</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
@@ -2092,62 +2086,62 @@
       </c>
       <c r="I29" s="11" t="inlineStr">
         <is>
-          <t>roles.id (ON DELETE CASCADE)</t>
+          <t>users.id (ON DELETE CASCADE)</t>
         </is>
       </c>
       <c r="J29" s="10" t="inlineStr"/>
       <c r="K29" s="11" t="inlineStr"/>
       <c r="L29" s="11" t="inlineStr">
         <is>
+          <t>회원 번호</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>user_roles</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>회원-역할 연결</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>role_id</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr"/>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
+        <is>
+          <t>roles.id (ON DELETE CASCADE)</t>
+        </is>
+      </c>
+      <c r="J30" s="10" t="inlineStr"/>
+      <c r="K30" s="11" t="inlineStr"/>
+      <c r="L30" s="11" t="inlineStr">
+        <is>
           <t>역할 번호</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>terms</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>약관</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G30" s="8" t="inlineStr">
-        <is>
-          <t>자동 증가</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="I30" s="8" t="inlineStr"/>
-      <c r="J30" s="6" t="inlineStr"/>
-      <c r="K30" s="8" t="inlineStr"/>
-      <c r="L30" s="8" t="inlineStr">
-        <is>
-          <t>약관 번호</t>
         </is>
       </c>
     </row>
@@ -2167,12 +2161,12 @@
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>VARCHAR(30)</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -2180,22 +2174,22 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G31" s="8" t="inlineStr"/>
-      <c r="H31" s="6" t="inlineStr"/>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>자동 증가</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="I31" s="8" t="inlineStr"/>
-      <c r="J31" s="6" t="inlineStr">
-        <is>
-          <t>복합(code, version)</t>
-        </is>
-      </c>
-      <c r="K31" s="8" t="inlineStr">
-        <is>
-          <t>UNIQUE terms_code_version_key</t>
-        </is>
-      </c>
+      <c r="J31" s="6" t="inlineStr"/>
+      <c r="K31" s="8" t="inlineStr"/>
       <c r="L31" s="8" t="inlineStr">
         <is>
-          <t>약관 코드 (terms / privacy / marketing)</t>
+          <t>약관 번호</t>
         </is>
       </c>
     </row>
@@ -2215,12 +2209,12 @@
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>INTEGER</t>
+          <t>VARCHAR(30)</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -2243,7 +2237,7 @@
       </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
-          <t>약관 버전. 문구가 바뀌면 새 행 추가</t>
+          <t>약관 코드 (terms / privacy / marketing)</t>
         </is>
       </c>
     </row>
@@ -2263,12 +2257,12 @@
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>version</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -2279,11 +2273,19 @@
       <c r="G33" s="8" t="inlineStr"/>
       <c r="H33" s="6" t="inlineStr"/>
       <c r="I33" s="8" t="inlineStr"/>
-      <c r="J33" s="6" t="inlineStr"/>
-      <c r="K33" s="8" t="inlineStr"/>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>복합(code, version)</t>
+        </is>
+      </c>
+      <c r="K33" s="8" t="inlineStr">
+        <is>
+          <t>UNIQUE terms_code_version_key</t>
+        </is>
+      </c>
       <c r="L33" s="8" t="inlineStr">
         <is>
-          <t>약관 제목</t>
+          <t>약관 버전. 문구가 바뀌면 새 행 추가</t>
         </is>
       </c>
     </row>
@@ -2303,12 +2305,12 @@
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>is_required</t>
+          <t>title</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>BOOLEAN</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -2323,7 +2325,7 @@
       <c r="K34" s="8" t="inlineStr"/>
       <c r="L34" s="8" t="inlineStr">
         <is>
-          <t>필수 동의 여부</t>
+          <t>약관 제목</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2345,7 @@
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>is_active</t>
+          <t>is_required</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -2356,18 +2358,14 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G35" s="8" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+      <c r="G35" s="8" t="inlineStr"/>
       <c r="H35" s="6" t="inlineStr"/>
       <c r="I35" s="8" t="inlineStr"/>
       <c r="J35" s="6" t="inlineStr"/>
       <c r="K35" s="8" t="inlineStr"/>
       <c r="L35" s="8" t="inlineStr">
         <is>
-          <t>현재 버전 여부 (가입 화면에 보이는 약관)</t>
+          <t>필수 동의 여부</t>
         </is>
       </c>
     </row>
@@ -2387,12 +2385,12 @@
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>is_active</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>TIMESTAMPTZ</t>
+          <t>BOOLEAN</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -2402,7 +2400,7 @@
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>now()</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr"/>
@@ -2411,55 +2409,51 @@
       <c r="K36" s="8" t="inlineStr"/>
       <c r="L36" s="8" t="inlineStr">
         <is>
+          <t>현재 버전 여부 (가입 화면에 보이는 약관)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>terms</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>약관</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr"/>
+      <c r="I37" s="8" t="inlineStr"/>
+      <c r="J37" s="6" t="inlineStr"/>
+      <c r="K37" s="8" t="inlineStr"/>
+      <c r="L37" s="8" t="inlineStr">
+        <is>
           <t>등록 시각</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="10" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>user_term_agreements</t>
-        </is>
-      </c>
-      <c r="C37" s="11" t="inlineStr">
-        <is>
-          <t>약관 동의 기록</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="inlineStr">
-        <is>
-          <t>user_id</t>
-        </is>
-      </c>
-      <c r="E37" s="11" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="F37" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G37" s="11" t="inlineStr"/>
-      <c r="H37" s="10" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="I37" s="11" t="inlineStr">
-        <is>
-          <t>users.id (ON DELETE CASCADE)</t>
-        </is>
-      </c>
-      <c r="J37" s="10" t="inlineStr"/>
-      <c r="K37" s="11" t="inlineStr"/>
-      <c r="L37" s="11" t="inlineStr">
-        <is>
-          <t>회원 번호</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2473,7 @@
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>term_id</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
@@ -2500,14 +2494,14 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>terms.id</t>
+          <t>users.id (ON DELETE CASCADE)</t>
         </is>
       </c>
       <c r="J38" s="10" t="inlineStr"/>
       <c r="K38" s="11" t="inlineStr"/>
       <c r="L38" s="11" t="inlineStr">
         <is>
-          <t>약관 번호 (버전 포함)</t>
+          <t>회원 번호</t>
         </is>
       </c>
     </row>
@@ -2527,12 +2521,12 @@
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>agreed_at</t>
+          <t>term_id</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
         <is>
-          <t>TIMESTAMPTZ</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="F39" s="10" t="inlineStr">
@@ -2540,66 +2534,66 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G39" s="11" t="inlineStr">
-        <is>
-          <t>now()</t>
-        </is>
-      </c>
-      <c r="H39" s="10" t="inlineStr"/>
-      <c r="I39" s="11" t="inlineStr"/>
+      <c r="G39" s="11" t="inlineStr"/>
+      <c r="H39" s="10" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="I39" s="11" t="inlineStr">
+        <is>
+          <t>terms.id</t>
+        </is>
+      </c>
       <c r="J39" s="10" t="inlineStr"/>
       <c r="K39" s="11" t="inlineStr"/>
       <c r="L39" s="11" t="inlineStr">
         <is>
+          <t>약관 번호 (버전 포함)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>user_term_agreements</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>약관 동의 기록</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>agreed_at</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="H40" s="10" t="inlineStr"/>
+      <c r="I40" s="11" t="inlineStr"/>
+      <c r="J40" s="10" t="inlineStr"/>
+      <c r="K40" s="11" t="inlineStr"/>
+      <c r="L40" s="11" t="inlineStr">
+        <is>
           <t>동의 시각</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>email_verifications</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>이메일 인증번호</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G40" s="8" t="inlineStr">
-        <is>
-          <t>자동 증가</t>
-        </is>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="I40" s="8" t="inlineStr"/>
-      <c r="J40" s="6" t="inlineStr"/>
-      <c r="K40" s="8" t="inlineStr"/>
-      <c r="L40" s="8" t="inlineStr">
-        <is>
-          <t>인증 기록 번호 (가입 증표 토큰에 들어감)</t>
         </is>
       </c>
     </row>
@@ -2619,12 +2613,12 @@
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>VARCHAR(255)</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
@@ -2632,18 +2626,22 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G41" s="8" t="inlineStr"/>
-      <c r="H41" s="6" t="inlineStr"/>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>자동 증가</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="I41" s="8" t="inlineStr"/>
       <c r="J41" s="6" t="inlineStr"/>
-      <c r="K41" s="8" t="inlineStr">
-        <is>
-          <t>ix_email_verifications_email</t>
-        </is>
-      </c>
+      <c r="K41" s="8" t="inlineStr"/>
       <c r="L41" s="8" t="inlineStr">
         <is>
-          <t>인증할 이메일</t>
+          <t>인증 기록 번호 (가입 증표 토큰에 들어감)</t>
         </is>
       </c>
     </row>
@@ -2663,12 +2661,12 @@
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>code_hash</t>
+          <t>email</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>VARCHAR(64)</t>
+          <t>VARCHAR(255)</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -2680,10 +2678,14 @@
       <c r="H42" s="6" t="inlineStr"/>
       <c r="I42" s="8" t="inlineStr"/>
       <c r="J42" s="6" t="inlineStr"/>
-      <c r="K42" s="8" t="inlineStr"/>
+      <c r="K42" s="8" t="inlineStr">
+        <is>
+          <t>ix_email_verifications_email</t>
+        </is>
+      </c>
       <c r="L42" s="8" t="inlineStr">
         <is>
-          <t>6자리 인증번호의 HMAC-SHA256 해시</t>
+          <t>인증할 이메일</t>
         </is>
       </c>
     </row>
@@ -2703,12 +2705,12 @@
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>expires_at</t>
+          <t>code_hash</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>TIMESTAMPTZ</t>
+          <t>VARCHAR(64)</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
@@ -2723,7 +2725,7 @@
       <c r="K43" s="8" t="inlineStr"/>
       <c r="L43" s="8" t="inlineStr">
         <is>
-          <t>인증번호 만료 시각 (발송 후 10분)</t>
+          <t>6자리 인증번호의 HMAC-SHA256 해시</t>
         </is>
       </c>
     </row>
@@ -2743,12 +2745,12 @@
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>attempts</t>
+          <t>expires_at</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>INTEGER</t>
+          <t>TIMESTAMPTZ</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -2756,18 +2758,14 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G44" s="8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="G44" s="8" t="inlineStr"/>
       <c r="H44" s="6" t="inlineStr"/>
       <c r="I44" s="8" t="inlineStr"/>
       <c r="J44" s="6" t="inlineStr"/>
       <c r="K44" s="8" t="inlineStr"/>
       <c r="L44" s="8" t="inlineStr">
         <is>
-          <t>틀린 횟수 (5회 이상이면 무효)</t>
+          <t>인증번호 만료 시각 (발송 후 10분)</t>
         </is>
       </c>
     </row>
@@ -2787,27 +2785,31 @@
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>verified_at</t>
+          <t>attempts</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>TIMESTAMPTZ</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G45" s="8" t="inlineStr"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="H45" s="6" t="inlineStr"/>
       <c r="I45" s="8" t="inlineStr"/>
       <c r="J45" s="6" t="inlineStr"/>
       <c r="K45" s="8" t="inlineStr"/>
       <c r="L45" s="8" t="inlineStr">
         <is>
-          <t>인증번호 확인 성공 시각</t>
+          <t>틀린 횟수 (5회 이상이면 무효)</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2829,7 @@
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>used_at</t>
+          <t>verified_at</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
@@ -2847,7 +2849,7 @@
       <c r="K46" s="8" t="inlineStr"/>
       <c r="L46" s="8" t="inlineStr">
         <is>
-          <t>가입(또는 이메일 변경)에 사용된 시각 (한 번만)</t>
+          <t>인증번호 확인 성공 시각</t>
         </is>
       </c>
     </row>
@@ -2867,7 +2869,7 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>used_at</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -2877,73 +2879,65 @@
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G47" s="8" t="inlineStr">
-        <is>
-          <t>now()</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr"/>
       <c r="H47" s="6" t="inlineStr"/>
       <c r="I47" s="8" t="inlineStr"/>
       <c r="J47" s="6" t="inlineStr"/>
-      <c r="K47" s="8" t="inlineStr">
+      <c r="K47" s="8" t="inlineStr"/>
+      <c r="L47" s="8" t="inlineStr">
+        <is>
+          <t>가입(또는 이메일 변경)에 사용된 시각 (한 번만)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>email_verifications</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>이메일 인증번호</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr"/>
+      <c r="I48" s="8" t="inlineStr"/>
+      <c r="J48" s="6" t="inlineStr"/>
+      <c r="K48" s="8" t="inlineStr">
         <is>
           <t>ix_email_verifications_created_at</t>
         </is>
       </c>
-      <c r="L47" s="8" t="inlineStr">
+      <c r="L48" s="8" t="inlineStr">
         <is>
           <t>발송 시각. 60초 간격·하루 10회 제한 계산, 7일 뒤 삭제</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="11" t="inlineStr">
-        <is>
-          <t>password_reset_tokens</t>
-        </is>
-      </c>
-      <c r="C48" s="11" t="inlineStr">
-        <is>
-          <t>비밀번호 재설정 토큰</t>
-        </is>
-      </c>
-      <c r="D48" s="11" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="E48" s="11" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="F48" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G48" s="11" t="inlineStr">
-        <is>
-          <t>자동 증가</t>
-        </is>
-      </c>
-      <c r="H48" s="10" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="I48" s="11" t="inlineStr"/>
-      <c r="J48" s="10" t="inlineStr"/>
-      <c r="K48" s="11" t="inlineStr"/>
-      <c r="L48" s="11" t="inlineStr">
-        <is>
-          <t>토큰 번호</t>
         </is>
       </c>
     </row>
@@ -2963,7 +2957,7 @@
       </c>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="E49" s="11" t="inlineStr">
@@ -2976,22 +2970,22 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G49" s="11" t="inlineStr"/>
-      <c r="H49" s="10" t="inlineStr"/>
-      <c r="I49" s="11" t="inlineStr">
-        <is>
-          <t>users.id (ON DELETE CASCADE)</t>
-        </is>
-      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>자동 증가</t>
+        </is>
+      </c>
+      <c r="H49" s="10" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="I49" s="11" t="inlineStr"/>
       <c r="J49" s="10" t="inlineStr"/>
-      <c r="K49" s="11" t="inlineStr">
-        <is>
-          <t>ix_password_reset_tokens_user_id</t>
-        </is>
-      </c>
+      <c r="K49" s="11" t="inlineStr"/>
       <c r="L49" s="11" t="inlineStr">
         <is>
-          <t>회원 번호</t>
+          <t>토큰 번호</t>
         </is>
       </c>
     </row>
@@ -3011,12 +3005,12 @@
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>token_hash</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>VARCHAR(64)</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="F50" s="10" t="inlineStr">
@@ -3026,20 +3020,20 @@
       </c>
       <c r="G50" s="11" t="inlineStr"/>
       <c r="H50" s="10" t="inlineStr"/>
-      <c r="I50" s="11" t="inlineStr"/>
-      <c r="J50" s="10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="I50" s="11" t="inlineStr">
+        <is>
+          <t>users.id (ON DELETE CASCADE)</t>
+        </is>
+      </c>
+      <c r="J50" s="10" t="inlineStr"/>
       <c r="K50" s="11" t="inlineStr">
         <is>
-          <t>UNIQUE password_reset_tokens_token_hash_key</t>
+          <t>ix_password_reset_tokens_user_id</t>
         </is>
       </c>
       <c r="L50" s="11" t="inlineStr">
         <is>
-          <t>링크 토큰의 HMAC-SHA256 해시 (원문은 메일로만)</t>
+          <t>회원 번호</t>
         </is>
       </c>
     </row>
@@ -3059,12 +3053,12 @@
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>expires_at</t>
+          <t>token_hash</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
         <is>
-          <t>TIMESTAMPTZ</t>
+          <t>VARCHAR(64)</t>
         </is>
       </c>
       <c r="F51" s="10" t="inlineStr">
@@ -3075,11 +3069,19 @@
       <c r="G51" s="11" t="inlineStr"/>
       <c r="H51" s="10" t="inlineStr"/>
       <c r="I51" s="11" t="inlineStr"/>
-      <c r="J51" s="10" t="inlineStr"/>
-      <c r="K51" s="11" t="inlineStr"/>
+      <c r="J51" s="10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K51" s="11" t="inlineStr">
+        <is>
+          <t>UNIQUE password_reset_tokens_token_hash_key</t>
+        </is>
+      </c>
       <c r="L51" s="11" t="inlineStr">
         <is>
-          <t>만료 시각 (발송 후 30분)</t>
+          <t>링크 토큰의 HMAC-SHA256 해시 (원문은 메일로만)</t>
         </is>
       </c>
     </row>
@@ -3099,7 +3101,7 @@
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>used_at</t>
+          <t>expires_at</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
@@ -3109,7 +3111,7 @@
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G52" s="11" t="inlineStr"/>
@@ -3119,7 +3121,7 @@
       <c r="K52" s="11" t="inlineStr"/>
       <c r="L52" s="11" t="inlineStr">
         <is>
-          <t>사용(또는 무효화) 시각</t>
+          <t>만료 시각 (발송 후 30분)</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3141,7 @@
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>used_at</t>
         </is>
       </c>
       <c r="E53" s="11" t="inlineStr">
@@ -3149,70 +3151,110 @@
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G53" s="11" t="inlineStr">
-        <is>
-          <t>now()</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G53" s="11" t="inlineStr"/>
       <c r="H53" s="10" t="inlineStr"/>
       <c r="I53" s="11" t="inlineStr"/>
       <c r="J53" s="10" t="inlineStr"/>
       <c r="K53" s="11" t="inlineStr"/>
       <c r="L53" s="11" t="inlineStr">
         <is>
+          <t>사용(또는 무효화) 시각</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>password_reset_tokens</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>비밀번호 재설정 토큰</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="E54" s="11" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="F54" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G54" s="11" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="H54" s="10" t="inlineStr"/>
+      <c r="I54" s="11" t="inlineStr"/>
+      <c r="J54" s="10" t="inlineStr"/>
+      <c r="K54" s="11" t="inlineStr"/>
+      <c r="L54" s="11" t="inlineStr">
+        <is>
           <t>발송 시각. 발송 횟수 제한 계산</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="6" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" s="8" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
         <is>
           <t>alembic_version</t>
         </is>
       </c>
-      <c r="C54" s="8" t="inlineStr">
+      <c r="C55" s="8" t="inlineStr">
         <is>
           <t>마이그레이션 버전</t>
         </is>
       </c>
-      <c r="D54" s="8" t="inlineStr">
+      <c r="D55" s="8" t="inlineStr">
         <is>
           <t>version_num</t>
         </is>
       </c>
-      <c r="E54" s="8" t="inlineStr">
+      <c r="E55" s="8" t="inlineStr">
         <is>
           <t>VARCHAR(32)</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G54" s="8" t="inlineStr"/>
-      <c r="H54" s="6" t="inlineStr">
+      <c r="G55" s="8" t="inlineStr"/>
+      <c r="H55" s="6" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="I54" s="8" t="inlineStr"/>
-      <c r="J54" s="6" t="inlineStr"/>
-      <c r="K54" s="8" t="inlineStr"/>
-      <c r="L54" s="8" t="inlineStr">
+      <c r="I55" s="8" t="inlineStr"/>
+      <c r="J55" s="6" t="inlineStr"/>
+      <c r="K55" s="8" t="inlineStr"/>
+      <c r="L55" s="8" t="inlineStr">
         <is>
           <t>현재 마이그레이션 리비전</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L54"/>
+  <autoFilter ref="A1:L55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(maemusae): 프로젝트 초대 (M2-1)
- mms_project_invitations 테이블: 토큰은 HMAC 해시만, 7일·1회, 같은 이메일 재초대 시 이전 초대 무효
  (살아 있는 초대는 프로젝트·이메일당 하나, 부분 유니크 인덱스). mms_project_members.invitation_id 추가
- 관리자 API: 초대 보내기(메일 mms_invite, BackgroundTasks)·대기 목록·취소
- 링크 API: lookup, signup-proof(킷 issue_verified_email_proof 로 인증번호 생략 가입 증표), accept(초대 이메일과 같은 계정만)
  토큰은 요청 로그에 남지 않도록 경로가 아니라 POST 본문으로 받음
- 없는·만료·취소·사용된 토큰은 모두 404 INVITATION_INVALID. 로그에는 초대 id 만
- 테이블 명세서, architecture.md, README 갱신. pytest 254

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AcRn9gV7oGMnFFhj3kFFXF
</commit_message>
<xml_diff>
--- a/docs/MeerKit_테이블명세서.xlsx
+++ b/docs/MeerKit_테이블명세서.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -513,6 +513,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -533,7 +534,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>24601a874fac</t>
+          <t>7b35839667fd</t>
         </is>
       </c>
     </row>
@@ -545,7 +546,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>feat/maemusae-m1 (매무새 프로젝트·멤버 추가)</t>
+          <t>feat/maemusae-invites (매무새 초대 추가)</t>
         </is>
       </c>
     </row>
@@ -557,7 +558,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25 (2026-10-27 users.avatar_key 추가, 2026-10-29 common_code_groups·common_codes, mms_projects·mms_project_members 추가). 소셜 로그인(social_accounts, users.has_password)은 아직 미반영</t>
+          <t>2026-10-25 (2026-10-27 users.avatar_key 추가, 2026-10-29 common_code_groups·common_codes, mms_projects·mms_project_members, mms_project_invitations·mms_project_members.invitation_id 추가). 소셜 로그인(social_accounts, users.has_password)은 아직 미반영</t>
         </is>
       </c>
     </row>
@@ -585,6 +586,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -869,7 +871,7 @@
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23">
@@ -878,31 +880,54 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>매무새 프로젝트 초대</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>프로젝트 관리자가 이메일로 보낸 초대. 토큰은 해시만, 7일·1회, 다시 초대하면 이전 초대 무효. 수락하면 멤버 행 추가</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
           <t>alembic_version</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>마이그레이션 버전</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>Alembic이 관리. 직접 수정하지 않음</t>
         </is>
       </c>
-      <c r="E23" s="6" t="n">
+      <c r="E24" s="6" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="24">
-      <c r="D24" s="2" t="inlineStr">
+    <row r="25">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="E24" s="9" t="n">
-        <v>83</v>
+      <c r="E25" s="9" t="n">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -916,7 +941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4495,31 +4520,31 @@
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>invitation_id</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
         <is>
-          <t>TIMESTAMPTZ</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G82" s="11" t="inlineStr">
-        <is>
-          <t>now()</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G82" s="11" t="n"/>
       <c r="H82" s="10" t="n"/>
-      <c r="I82" s="11" t="n"/>
+      <c r="I82" s="11" t="inlineStr">
+        <is>
+          <t>mms_project_invitations.id</t>
+        </is>
+      </c>
       <c r="J82" s="10" t="n"/>
       <c r="K82" s="11" t="n"/>
       <c r="L82" s="11" t="inlineStr">
         <is>
-          <t>만든 시각</t>
+          <t>초대로 들어온 멤버면 그 초대 (만든 사람은 비움). 초대 행이 지워지면 NULL (fk_mms_project_members_invitation_id)</t>
         </is>
       </c>
     </row>
@@ -4539,7 +4564,7 @@
       </c>
       <c r="D83" s="11" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="E83" s="11" t="inlineStr">
@@ -4563,49 +4588,573 @@
       <c r="K83" s="11" t="n"/>
       <c r="L83" s="11" t="inlineStr">
         <is>
+          <t>만든 시각</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="11" t="inlineStr">
+        <is>
+          <t>mms_project_members</t>
+        </is>
+      </c>
+      <c r="C84" s="11" t="inlineStr">
+        <is>
+          <t>매무새 프로젝트 멤버</t>
+        </is>
+      </c>
+      <c r="D84" s="11" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="E84" s="11" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="F84" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G84" s="11" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="H84" s="10" t="n"/>
+      <c r="I84" s="11" t="n"/>
+      <c r="J84" s="10" t="n"/>
+      <c r="K84" s="11" t="n"/>
+      <c r="L84" s="11" t="inlineStr">
+        <is>
           <t>마지막 수정 시각</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="6" t="n">
-        <v>83</v>
-      </c>
-      <c r="B84" s="8" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="10" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="11" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="C85" s="11" t="inlineStr">
+        <is>
+          <t>매무새 프로젝트 초대</t>
+        </is>
+      </c>
+      <c r="D85" s="11" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E85" s="11" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="F85" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G85" s="11" t="inlineStr">
+        <is>
+          <t>자동 증가</t>
+        </is>
+      </c>
+      <c r="H85" s="10" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="I85" s="11" t="n"/>
+      <c r="J85" s="10" t="n"/>
+      <c r="K85" s="11" t="n"/>
+      <c r="L85" s="11" t="inlineStr">
+        <is>
+          <t>초대 번호 (취소 API 경로에 씀)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="11" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="C86" s="11" t="inlineStr">
+        <is>
+          <t>매무새 프로젝트 초대</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="inlineStr">
+        <is>
+          <t>project_id</t>
+        </is>
+      </c>
+      <c r="E86" s="11" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="F86" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G86" s="11" t="n"/>
+      <c r="H86" s="10" t="n"/>
+      <c r="I86" s="11" t="inlineStr">
+        <is>
+          <t>mms_projects.id</t>
+        </is>
+      </c>
+      <c r="J86" s="10" t="inlineStr">
+        <is>
+          <t>Y (project_id, email) 살아 있는 초대만</t>
+        </is>
+      </c>
+      <c r="K86" s="11" t="n"/>
+      <c r="L86" s="11" t="inlineStr">
+        <is>
+          <t>프로젝트. 프로젝트 행이 지워지면 같이 삭제</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="11" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="C87" s="11" t="inlineStr">
+        <is>
+          <t>매무새 프로젝트 초대</t>
+        </is>
+      </c>
+      <c r="D87" s="11" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E87" s="11" t="inlineStr">
+        <is>
+          <t>VARCHAR(255)</t>
+        </is>
+      </c>
+      <c r="F87" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G87" s="11" t="n"/>
+      <c r="H87" s="10" t="n"/>
+      <c r="I87" s="11" t="n"/>
+      <c r="J87" s="10" t="inlineStr">
+        <is>
+          <t>Y (project_id, email) 살아 있는 초대만</t>
+        </is>
+      </c>
+      <c r="K87" s="11" t="inlineStr">
+        <is>
+          <t>ix_mms_project_invitations_email</t>
+        </is>
+      </c>
+      <c r="L87" s="11" t="inlineStr">
+        <is>
+          <t>초대받은 이메일 (소문자 저장). 로그에 남기지 않음</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="10" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="11" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="C88" s="11" t="inlineStr">
+        <is>
+          <t>매무새 프로젝트 초대</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="E88" s="11" t="inlineStr">
+        <is>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="F88" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G88" s="11" t="n"/>
+      <c r="H88" s="10" t="n"/>
+      <c r="I88" s="11" t="n"/>
+      <c r="J88" s="10" t="n"/>
+      <c r="K88" s="11" t="n"/>
+      <c r="L88" s="11" t="inlineStr">
+        <is>
+          <t>수락하면 받을 역할 ADMIN/MEMBER. CHECK (ck_mms_project_invitations_role)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="10" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="11" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="C89" s="11" t="inlineStr">
+        <is>
+          <t>매무새 프로젝트 초대</t>
+        </is>
+      </c>
+      <c r="D89" s="11" t="inlineStr">
+        <is>
+          <t>token_hash</t>
+        </is>
+      </c>
+      <c r="E89" s="11" t="inlineStr">
+        <is>
+          <t>VARCHAR(64)</t>
+        </is>
+      </c>
+      <c r="F89" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G89" s="11" t="n"/>
+      <c r="H89" s="10" t="n"/>
+      <c r="I89" s="11" t="n"/>
+      <c r="J89" s="10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K89" s="11" t="n"/>
+      <c r="L89" s="11" t="inlineStr">
+        <is>
+          <t>링크 토큰의 HMAC 해시 (core.security.hash_secret). 원문은 메일에만</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="10" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="11" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="C90" s="11" t="inlineStr">
+        <is>
+          <t>매무새 프로젝트 초대</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="inlineStr">
+        <is>
+          <t>invited_by</t>
+        </is>
+      </c>
+      <c r="E90" s="11" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="F90" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G90" s="11" t="n"/>
+      <c r="H90" s="10" t="n"/>
+      <c r="I90" s="11" t="inlineStr">
+        <is>
+          <t>users.id</t>
+        </is>
+      </c>
+      <c r="J90" s="10" t="n"/>
+      <c r="K90" s="11" t="n"/>
+      <c r="L90" s="11" t="inlineStr">
+        <is>
+          <t>초대한 프로젝트 관리자</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="11" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="C91" s="11" t="inlineStr">
+        <is>
+          <t>매무새 프로젝트 초대</t>
+        </is>
+      </c>
+      <c r="D91" s="11" t="inlineStr">
+        <is>
+          <t>expires_at</t>
+        </is>
+      </c>
+      <c r="E91" s="11" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="F91" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G91" s="11" t="n"/>
+      <c r="H91" s="10" t="n"/>
+      <c r="I91" s="11" t="n"/>
+      <c r="J91" s="10" t="n"/>
+      <c r="K91" s="11" t="n"/>
+      <c r="L91" s="11" t="inlineStr">
+        <is>
+          <t>만료 시각 (보낸 때 + 7일)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="10" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="11" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="C92" s="11" t="inlineStr">
+        <is>
+          <t>매무새 프로젝트 초대</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="inlineStr">
+        <is>
+          <t>accepted_at</t>
+        </is>
+      </c>
+      <c r="E92" s="11" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="F92" s="10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G92" s="11" t="n"/>
+      <c r="H92" s="10" t="n"/>
+      <c r="I92" s="11" t="n"/>
+      <c r="J92" s="10" t="n"/>
+      <c r="K92" s="11" t="n"/>
+      <c r="L92" s="11" t="inlineStr">
+        <is>
+          <t>수락 시각. 값이 있으면 다시 못 씀 (1회)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="11" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="C93" s="11" t="inlineStr">
+        <is>
+          <t>매무새 프로젝트 초대</t>
+        </is>
+      </c>
+      <c r="D93" s="11" t="inlineStr">
+        <is>
+          <t>accepted_user_id</t>
+        </is>
+      </c>
+      <c r="E93" s="11" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="F93" s="10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G93" s="11" t="n"/>
+      <c r="H93" s="10" t="n"/>
+      <c r="I93" s="11" t="inlineStr">
+        <is>
+          <t>users.id</t>
+        </is>
+      </c>
+      <c r="J93" s="10" t="n"/>
+      <c r="K93" s="11" t="n"/>
+      <c r="L93" s="11" t="inlineStr">
+        <is>
+          <t>수락한 회원</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="10" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="11" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="C94" s="11" t="inlineStr">
+        <is>
+          <t>매무새 프로젝트 초대</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="inlineStr">
+        <is>
+          <t>revoked_at</t>
+        </is>
+      </c>
+      <c r="E94" s="11" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="F94" s="10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G94" s="11" t="n"/>
+      <c r="H94" s="10" t="n"/>
+      <c r="I94" s="11" t="n"/>
+      <c r="J94" s="10" t="n"/>
+      <c r="K94" s="11" t="n"/>
+      <c r="L94" s="11" t="inlineStr">
+        <is>
+          <t>취소 시각 (관리자가 취소하거나 같은 이메일로 다시 초대하면 기록)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="10" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="11" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="C95" s="11" t="inlineStr">
+        <is>
+          <t>매무새 프로젝트 초대</t>
+        </is>
+      </c>
+      <c r="D95" s="11" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="E95" s="11" t="inlineStr">
+        <is>
+          <t>TIMESTAMPTZ</t>
+        </is>
+      </c>
+      <c r="F95" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G95" s="11" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="H95" s="10" t="n"/>
+      <c r="I95" s="11" t="n"/>
+      <c r="J95" s="10" t="n"/>
+      <c r="K95" s="11" t="n"/>
+      <c r="L95" s="11" t="inlineStr">
+        <is>
+          <t>보낸 시각 (대기 목록 정렬)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
         <is>
           <t>alembic_version</t>
         </is>
       </c>
-      <c r="C84" s="8" t="inlineStr">
+      <c r="C96" s="8" t="inlineStr">
         <is>
           <t>마이그레이션 버전</t>
         </is>
       </c>
-      <c r="D84" s="8" t="inlineStr">
+      <c r="D96" s="8" t="inlineStr">
         <is>
           <t>version_num</t>
         </is>
       </c>
-      <c r="E84" s="8" t="inlineStr">
+      <c r="E96" s="8" t="inlineStr">
         <is>
           <t>VARCHAR(32)</t>
         </is>
       </c>
-      <c r="F84" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G84" s="8" t="inlineStr"/>
-      <c r="H84" s="6" t="inlineStr">
+      <c r="F96" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G96" s="8" t="inlineStr"/>
+      <c r="H96" s="6" t="inlineStr">
         <is>
           <t>PK</t>
         </is>
       </c>
-      <c r="I84" s="8" t="inlineStr"/>
-      <c r="J84" s="6" t="inlineStr"/>
-      <c r="K84" s="8" t="inlineStr"/>
-      <c r="L84" s="8" t="inlineStr">
+      <c r="I96" s="8" t="inlineStr"/>
+      <c r="J96" s="6" t="inlineStr"/>
+      <c r="K96" s="8" t="inlineStr"/>
+      <c r="L96" s="8" t="inlineStr">
         <is>
           <t>현재 마이그레이션 리비전</t>
         </is>
@@ -4623,7 +5172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4986,9 +5535,136 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>project_id</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>mms_projects.id</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>N:1</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>CASCADE</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>프로젝트 행이 지워지면 초대도 삭제</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>invited_by</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>users.id</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>N:1</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>제한(NO ACTION)</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>초대한 사람 (회원은 실제로 지우지 않음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>mms_project_invitations</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>accepted_user_id</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>users.id</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>N:1</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>제한(NO ACTION)</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>수락한 회원</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>mms_project_members</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>invitation_id</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>mms_project_invitations.id</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>N:1 (선택)</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>SET NULL</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>초대로 들어온 멤버. 초대가 지워져도 멤버는 남음</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>참고: 회원은 실제로 지우지 않고(탈퇴는 deactivated_at, 365일 뒤 개인정보만 파기), 행을 남겨 다른 데이터의 참조가 깨지지 않게 합니다.</t>
         </is>

</xml_diff>